<commit_message>
Add GUIDED SEMISUPERVISED TM
</commit_message>
<xml_diff>
--- a/out/taxonomy_comparison.xlsx
+++ b/out/taxonomy_comparison.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E52"/>
+  <dimension ref="A1:E53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -457,20 +457,20 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>bitcoin vendere portafoglio conio _x00d connessione inviare invio sezione limite</t>
+          <t>truffa stato pagamento truffato sicurezza soldi dopo hacker rimborso modulo</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>problemi_bitcoin</t>
+          <t>problemi_sicurezza</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>0.7041000127792358</v>
+        <v>0.6894999742507935</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -480,20 +480,20 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>34</v>
+        <v>13</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>contanti ricarica opzione cashback ricariche disponibile costosi rimborsano 77 46</t>
+          <t>assistenza servizio assente pessima scadente assistenza_inesistente scarsa peggiore totalmente assistenti</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>problemi_cashback</t>
+          <t>problemi_assistenza</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>0.6990000009536743</v>
+        <v>0.6686999797821045</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -503,11 +503,11 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>servizio_clienti inesistente clienti pessimo cliente veramente assistenza pessima supporto esiste</t>
+          <t>servizio_clienti inesistente cliente assistenza criticità significativi esiste evidenziando risponde assenza</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -516,7 +516,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>0.6800000071525574</v>
+        <v>0.6636999845504761</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -526,20 +526,20 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>truffa phishing truffato denuncia hacker numero brutta carabinieri operazione attacco</t>
+          <t>accesso_biometrico valido biometrico riconoscimento segnalo problemi accesso accedere login spesso</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>problemi_sicurezza</t>
+          <t>problemi_accesso</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>0.671999990940094</v>
+        <v>0.6417000293731689</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -549,20 +549,20 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>assistenza inesistente assente totalmente zero risolvere pessima importanti desiderare assistenza_inesistente</t>
+          <t>bitcoin vendere portafoglio conio connessione _x00d acquistare inviare invio euro</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>problemi_assistenza</t>
+          <t>problemi_bitcoin</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>0.6363999843597412</v>
+        <v>0.629800021648407</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -572,20 +572,20 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>29</v>
+        <v>46</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>paypal pagamenti_online trasferimento pagamento_online pausa x00d confermare attiva _x00d carta</t>
+          <t>confermare pagamenti_online transazione codice acquisto pagamento pagamento_online conferma notifica corretto</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>problemi_circuiti_pagamento</t>
+          <t>problemi_pagamenti_online</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>0.6118999719619751</v>
+        <v>0.6013000011444092</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -595,20 +595,20 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>22</v>
+        <v>6</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>registrarmi dati registrarsi errore registrazione impossibile errori corretti errati pagina</t>
+          <t>carta nuova ricaricare carta_fisica posta altra pessimo arrivata pagato ricarica</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>problemi_dati_conto</t>
+          <t>problemi_ricarica</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>0.5900999903678894</v>
+        <v>0.5960000157356262</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -618,20 +618,20 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>euro 25 50 bonus mese ricevuto invito codice spariti regalo</t>
+          <t>dati registrarmi registrazione giusti registrarsi errore dice registrare corretti errati</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>problemi_concorsi_bonus</t>
+          <t>problemi_registrazione</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>0.5776000022888184</v>
+        <v>0.5898000001907349</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -641,20 +641,20 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>35</v>
+        <v>22</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>telefonica numero telefonico cellulare assistenza associare annullare cercate serie parlare</t>
+          <t>accesso accedere va riesce caricamento apre fa riesci problemi oggi</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>problemi_ricarica_telefonica</t>
+          <t>problemi_accesso</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>0.553600013256073</v>
+        <v>0.5879999995231628</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -664,47 +664,47 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>7</v>
+        <v>47</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>_x00d prodotto assistenza italia servizi commissioni stata nonostante cliente accredito</t>
+          <t>permessi pagamenti ricevute scaricare pagamento riesco permette line on quant</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>problemi_servizi_partner</t>
+          <t>problemi_circuiti_pagamento</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>0.5371000170707703</v>
+        <v>0.5629000067710876</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Weak/New</t>
+          <t>Strong</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>37</v>
+        <v>1</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>credito credit boost carte addebiti urgentemente succede dà aumenta apposto</t>
+          <t>password cambiare errore entrare errata continua accesso dice login creare</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>problemi_sezione_credito</t>
+          <t>problemi_accesso</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>0.5364999771118164</v>
+        <v>0.5616999864578247</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Weak/New</t>
+          <t>Strong</t>
         </is>
       </c>
     </row>
@@ -714,85 +714,85 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>crash crasha movimenti troppi edit appena continui inutilizzabile spesso mollo</t>
+          <t>storto andato qualcosa messaggio ops correttamente accedere _x00d x00d app_x00d</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>problemi_risparmi</t>
+          <t>problemi_accesso</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>0.5353999733924866</v>
+        <v>0.5558000206947327</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Weak/New</t>
+          <t>Strong</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>notifiche pubblicità spam disattivare promozioni suono promozionali notifiche_push notifica notifiche_pubblicitarie</t>
+          <t>bonus euro promozione promo codice 25 20 invito mese accreditato</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>problemi_comunicazione</t>
+          <t>problemi_concorsi_bonus</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>0.5120000243186951</v>
+        <v>0.5550000071525574</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Weak/New</t>
+          <t>Strong</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>43</v>
+        <v>4</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>aggiornamenti aggiorna ultimi aggiornarla upgrade rettifico risolvano automatici udite viste</t>
+          <t>bug spesso accesso continui crash veramente problemi troppi thumbs_down pessima</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>problemi_aggiornamento_app</t>
+          <t>problemi_risparmi</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>0.4939999878406525</v>
+        <v>0.5515999794006348</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Weak/New</t>
+          <t>Strong</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>33</v>
+        <v>7</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>box risparmi sezione risparmio fondi prelievo data uscite mensile movimenti</t>
+          <t>funziona soldi pagamenti servizio accedere volte così estero tanto servizi</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>problemi_risparmi</t>
+          <t>problemi_pagamenti_carta</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>0.4611000120639801</v>
+        <v>0.5254999995231628</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -802,20 +802,20 @@
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>21</v>
+        <v>5</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>andato qualcosa storto ops errori troppi errore finito ultimamente moglie</t>
+          <t>notifiche pubblicità spam promozioni disattivare notifiche_push notifiche_pubblicitarie troppa arrivano possono</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>problemi_chiusura_conto</t>
+          <t>problemi_comunicazione</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>0.4589999914169312</v>
+        <v>0.5113999843597412</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -825,20 +825,20 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>password cambiare login errore cambio cambiato impronta inserire credenziali metto</t>
+          <t>android samsung compatibile versione smartphone crasha ultimo operativo aggiornamento dopo</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>problemi_accesso</t>
+          <t>problemi_download_app</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>0.4589000046253204</v>
+        <v>0.5109000205993652</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -848,20 +848,20 @@
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>lenta diventata lentezza caricamenti pesante contenuto lentissimo avviarsi pò volte</t>
+          <t>notifiche notifiche_pubblicitarie suono disattivare promozionali pubblicità buona fastidiose android molto</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>problemi_prelievi</t>
+          <t>problemi_comunicazione</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>0.4449999928474426</v>
+        <v>0.5074999928474426</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -871,20 +871,20 @@
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>1</v>
+        <v>44</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>carta carta_fisica ricaricare altra ricarica scadenza dati mese arrivata nn</t>
+          <t>assistenza 48 contattare reparto ore servizio competente impossibile pagando nè</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>problemi_ricarica</t>
+          <t>problemi_assistenza</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>0.4352000057697296</v>
+        <v>0.5069000124931335</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -894,20 +894,20 @@
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>36</v>
+        <v>8</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>motivazioni idoneo riferimento fonti nexi apertura presenza pubblicamente fase diniego</t>
+          <t>aggiornamento ultimo dopo aggiorna aggiornamenti versione accede funziona rubrica continua</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>problemi_comunicazione</t>
+          <t>problemi_aggiornamento_app</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>0.4345000088214874</v>
+        <v>0.5042999982833862</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -917,20 +917,20 @@
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>chiude chiudere blocca retrocedere sola piano ultimo continua motivo appena</t>
+          <t>banche sella italia assistenza altra mai esperienza bank così servizio</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>problemi_blocco_conto_af</t>
+          <t>problemi_sezione_credito</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>0.4289000034332275</v>
+        <v>0.5041999816894531</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -940,20 +940,20 @@
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>ore 48 risposta email entro nessuna giorni servizio_clienti via risponde</t>
+          <t>contanti pagamenti ricaricare tornerà succedere ricariche ricarica premium costo abbonamento</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>problemi_registrazione</t>
+          <t>problemi_cashback</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>0.4284000098705292</v>
+        <v>0.501800000667572</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -963,20 +963,20 @@
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>40</v>
+        <v>3</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>google play playstore pay store wallet aggiornarla riuscivo saputo aggiungere</t>
+          <t>password accedere cambiare accesso cambio entrare né errore riesco dopo</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>problemi_pagamenti_carta</t>
+          <t>problemi_accesso</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>0.4271999895572662</v>
+        <v>0.5006999969482422</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -986,11 +986,11 @@
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>accesso_biometrico valido biometrico segnalo riconoscimento login spesso messaggio biometria innovativa</t>
+          <t>account riesco accedere profilo web accesso entrare giorni sito problemi</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -999,7 +999,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>0.4187999963760376</v>
+        <v>0.4932000041007996</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -1009,20 +1009,20 @@
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>42</v>
+        <v>0</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>pessima veramente pessimo peggio bonifico nega thumbs_down malissimo peggior larga</t>
+          <t>chat operatore parlare bot assistenza mail servizio_clienti rispondono via contattare</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>problemi_chiusura_conto</t>
+          <t>problemi_comunicazione</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>0.4178999960422516</v>
+        <v>0.4815999865531921</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -1032,20 +1032,20 @@
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>41</v>
+        <v>21</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>email mail nessuno perche risponde nulla nessuna acquisto scrivo apre</t>
+          <t>carta riesco posso appena carta_fisica apre fa scarico usare accedere</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>problemi_invio_denaro_hypers</t>
+          <t>problemi_gestione_carta</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>0.4153999984264374</v>
+        <v>0.480100005865097</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1055,20 +1055,20 @@
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>3</v>
+        <v>38</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>chat operatore bot parlare minuti assistenza chatbot ore risponde attesa</t>
+          <t>amazon acquisto pagamento carta qui ordine instagram pagare ve mai</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>problemi_comunicazione</t>
+          <t>problemi_pagamenti_carta</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>0.4083999991416931</v>
+        <v>0.4785999953746796</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1078,20 +1078,20 @@
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>bloccata carta blocco avviso bloccato ticket email stata ripetute dicono</t>
+          <t>soldi pagamento stato bonifico bloccato anno me rimborso macchina sicuramente</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>problemi_blocco_conto_af</t>
+          <t>problemi_cashback</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>0.4043999910354614</v>
+        <v>0.4593000113964081</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -1101,20 +1101,20 @@
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>31</v>
+        <v>48</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>figlio registrazione minorenne genitore attivazione minorenni figlia gg documenti mail</t>
+          <t>costo mese 90 paypal gratuita pagamenti funziona spazi permetta infinite</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>problemi_registrazione</t>
+          <t>problemi_pagamenti_carta</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>0.3987999856472015</v>
+        <v>0.449999988079071</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1124,20 +1124,20 @@
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>android samsung folded_hands compatibile smartphone pro crasha ultimo lg pixel</t>
+          <t>lenta troppo secondi lentezza lento lentissima avviarsi caricamento molto macchinosa</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>problemi_download_app</t>
+          <t>problemi_chiusura_conto</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>0.3971000015735626</v>
+        <v>0.448500007390976</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1147,20 +1147,20 @@
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>46</v>
+        <v>32</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>scaricare permessi ricevute oppo reno giacenza consente ricevuta download nn</t>
+          <t>box risparmi folded_hands prelievo sezione movimenti conio bene esperienza trovo</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>problemi_download_app</t>
+          <t>problemi_risparmi</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>0.3853000104427338</v>
+        <v>0.443699985742569</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1170,20 +1170,20 @@
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>28</v>
+        <v>49</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>ultimo ultima apre uscire chiudere presto sbatte grossa release macchinoso</t>
+          <t>whatsapp premium risposta numero attivi dovrebbe messaggio assistenza attesa chat</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>problemi_chiusura_conto</t>
+          <t>problemi_comunicazione</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>0.3781999945640564</v>
+        <v>0.414000004529953</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1193,20 +1193,20 @@
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>39</v>
+        <v>2</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>venditore merce _x00d modulo contabilizzate clown_face verso importo x00d operatrice</t>
+          <t>aggiornamento aggiornare store ultimo versione aggiorna scaricare apre dice play</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>problemi_concorsi_bonus</t>
+          <t>problemi_aggiornamento_app</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>0.3659999966621399</v>
+        <v>0.4135999977588654</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1216,20 +1216,20 @@
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>15</v>
+        <v>34</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>face id accesso_biometrico grinning_face_with_sweat apre clown_face manualmente riconosce valido loop</t>
+          <t>email carta dopo documento senza richiesta stata bloccato ticket rifiuto</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>problemi_accesso</t>
+          <t>problemi_registrazione</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>0.3580000102519989</v>
+        <v>0.4009000062942505</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1239,20 +1239,20 @@
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>49</v>
+        <v>29</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>bagga rapidamente rivedere riprovo smesso poi volevo completamente crash funzionare</t>
+          <t>ios iphone 12 aggiornamento ultimo crash apre versione entrata 13</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>problemi_disponibilità</t>
+          <t>problemi_download_app</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>0.3555000126361847</v>
+        <v>0.3837999999523163</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -1262,20 +1262,20 @@
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>whatsapp premium attivi veniva numero assistenza direttamente dedicato rispondere dovrebbe</t>
+          <t>numero opzione vergognosa and logicamente cambiato professionali pensato invio chiamare</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>problemi_comunicazione</t>
+          <t>problemi_upgrade</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>0.3388000130653381</v>
+        <v>0.380299985408783</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1285,20 +1285,20 @@
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>10</v>
+        <v>41</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>sms codice arriva verifica messaggio ops codici storto via andato</t>
+          <t>conferma registrazione ancora arrivata email 08 mandato giorni 23 entro</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>problemi_ricarica_telefonica</t>
+          <t>problemi_registrazione</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>0.3348999917507172</v>
+        <v>0.3770000040531158</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1308,11 +1308,11 @@
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>video foto documento registrazione identità documenti file registrare arrivo provo</t>
+          <t>video documento foto identità registrazione riconoscimento registrare documenti immagini rifiutato</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1321,7 +1321,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>0.3325000107288361</v>
+        <v>0.3714999854564667</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1331,20 +1331,20 @@
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>5</v>
+        <v>40</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>ciao permette tanto caricare bonifici truffatori risolvere altro accedo mette</t>
+          <t>accedere funziona aggiornata posso accedo dispositivo provo programma contattarvi apre</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>problemi_chiusura_conto</t>
+          <t>problemi_download_app</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>0.3253999948501587</v>
+        <v>0.3714999854564667</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1354,20 +1354,20 @@
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>25</v>
+        <v>11</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>soggiorno postale permesso 02 codice seguito 16 poliziotto prefisso già</t>
+          <t>face id riconoscimento riconosce facciale accesso_biometrico volto funziona iphone accedere</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>problemi_sicurezza</t>
+          <t>problemi_accesso</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>0.314300000667572</v>
+        <v>0.3695000112056732</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1377,20 +1377,20 @@
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>44</v>
+        <v>26</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>bonifici_istantanei sella gruppo illimity bonifici_istantaneo bonifici unicredit arrivano finalmente entrata</t>
+          <t>lenta molto diventata caricamenti sezioni lentezza apertura carina pò varie</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>problemi_concorsi_bonus</t>
+          <t>problemi_prelievi</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>0.3041000068187714</v>
+        <v>0.3630000054836273</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1400,11 +1400,11 @@
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>12</v>
+        <v>33</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>reinstallare disinstallare installare apre reinstallata disinstallata reinstallato disinstallato disinstallando reinstallando</t>
+          <t>soldi contanti box effettuo risparmio down immediato me altrove devo</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1413,7 +1413,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>0.298799991607666</v>
+        <v>0.3431999981403351</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1423,20 +1423,20 @@
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>8</v>
+        <v>37</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>iphone ios 12 ultimo apple crash riconosce id pro apre</t>
+          <t>riesco entrare accedere ciao nessun prevista immensa my impossibile permette</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>problemi_download_app</t>
+          <t>problemi_invio_denaro_hypers</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>0.2930999994277954</v>
+        <v>0.3397000133991241</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1446,20 +1446,20 @@
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>27</v>
+        <v>50</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>amazon acquisto carta qui instagram ordine ve chiedete farvi devi</t>
+          <t>funziona funzionano emolumento bonifico va 07 scarico cliccare traccia 31</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>problemi_pagamenti_carta</t>
+          <t>problemi_ricarica</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>0.2865000069141388</v>
+        <v>0.3276000022888184</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1469,20 +1469,20 @@
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>26</v>
+        <v>51</v>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>bonifici aderire pieta tratti pianta lapp servito buttati alte lenta</t>
+          <t>telefono arriva mps riceverò telefoniche messaggio nuovo associare via wifi</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>problemi_lista_movimenti</t>
+          <t>problemi_ricarica_telefonica</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>0.2788000106811523</v>
+        <v>0.3228999972343445</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -1492,20 +1492,20 @@
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>38</v>
+        <v>10</v>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t xml:space="preserve">         </t>
+          <t>chiude apre appena aggiornamento ultimo dopo aprire potete sola apro</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>problemi_chiusura_conto</t>
+          <t>problemi_aggiornamento_app</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>0.2644999921321869</v>
+        <v>0.3012000024318695</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -1515,20 +1515,20 @@
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>ricaricare tabacchino contanti tabaccaio qr tabacchi poi ossia pensate tabaccheria</t>
+          <t>sms codice arriva verifica via arrivano accedere codici inserire mai</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>problemi_blocco_conto_af</t>
+          <t>problemi_accesso</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>0.2558000087738037</v>
+        <v>0.2931999862194061</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -1538,20 +1538,20 @@
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>apre aprire sì 22 potete subito aprirsi risolvere tante 26</t>
+          <t>cattivo bha puro spiegate emettere schifo revolut tratti fidatevi instantaneo</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>problemi_f24</t>
+          <t>problemi_blocco_conto_af</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>0.2471999973058701</v>
+        <v>0.2540000081062317</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1561,20 +1561,20 @@
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>impossibile nulla niente nemmeno né no potevano robot riesce sconsigliata</t>
+          <t>entrare giorni riuscivo settimana riesco accedere fa provo aprirmi playstore</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>problemi_sistema</t>
+          <t>problemi_concorsi_bonus</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>0.2221000045537949</v>
+        <v>0.2410999983549118</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -1584,20 +1584,20 @@
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>18</v>
+        <v>36</v>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>stelle do stella mettere dato it quattro poter zero due</t>
+          <t>giorni riesco due andata carica funzionato fine inizio settimana mesi</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>problemi_ricarica</t>
+          <t>problemi_disponibilità</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>0.2108999937772751</v>
+        <v>0.2194000035524368</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -1607,22 +1607,45 @@
     </row>
     <row r="52">
       <c r="A52" t="n">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>giorni giorno due qualche tre provo eternità niente disservizio carica</t>
+          <t>fa bonifici capisco retrocedere piano indietro revolut assurdo ce tasto</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>problemi_disponibilità</t>
+          <t>problemi_chiusura_conto</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>0.1841000020503998</v>
+        <v>0.2030999958515167</v>
       </c>
       <c r="E52" t="inlineStr">
+        <is>
+          <t>Weak/New</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>25</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>stelle stella questionario do tolgo dato mettere plafond ottimo settimana</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>problemi_concorsi_bonus</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>0.1805000007152557</v>
+      </c>
+      <c r="E53" t="inlineStr">
         <is>
           <t>Weak/New</t>
         </is>

</xml_diff>

<commit_message>
Add draft for LLM topic representations
</commit_message>
<xml_diff>
--- a/out/taxonomy_comparison.xlsx
+++ b/out/taxonomy_comparison.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -457,20 +457,20 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>carta dopo mai senza fa soldi problema problemi riesco accedere</t>
+          <t xml:space="preserve"> Problemi di assistenza scadente         </t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>problemi_upgrade</t>
+          <t>problemi_assistenza</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>0.9287999868392944</v>
+        <v>0.7742999792098999</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -480,20 +480,20 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>stelle giorni fa accedere ormai do resto entrare anno settimane</t>
+          <t xml:space="preserve"> Problemi di accesso all'app.         </t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>problemi_upgrade</t>
+          <t>problemi_accesso</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>0.9229000210762024</v>
+        <v>0.7681999802589417</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -503,20 +503,20 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>accedere riesco fa entrare carta password giorni problema problemi quando</t>
+          <t xml:space="preserve"> Problemi di accesso all'app             </t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>problemi_upgrade</t>
+          <t>problemi_accesso</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>0.9003000259399414</v>
+        <v>0.7448999881744385</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -526,20 +526,20 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>lenta impossibile troppo notifiche blocca ricarica pagamenti funziona lentissima bonifici</t>
+          <t xml:space="preserve"> Problemi di pagamento.         </t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>problemi_upgrade</t>
+          <t>problemi_circuiti_pagamento</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>0.885200023651123</v>
+        <v>0.7391999959945679</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -549,20 +549,20 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>enraged_face davvero devo registrazione cosa ogni clown_face carta assistenza apre</t>
+          <t xml:space="preserve"> Problemi di pagamento.         </t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>problemi_upgrade</t>
+          <t>problemi_circuiti_pagamento</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>0.8636999726295471</v>
+        <v>0.7391999959945679</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -572,20 +572,21 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>assistenza inesistente scarsa assente contattare wathsapp insoddisfatto clienti fornisce penosa</t>
+          <t xml:space="preserve">
+Problemi di accesso al         </t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>problemi_assistenza</t>
+          <t>problemi_accesso</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>0.8235999941825867</v>
+        <v>0.7376000285148621</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -595,20 +596,20 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>account codice difficile pubblicità riesco stato chiudere privacy trasferimento utilizzato</t>
+          <t xml:space="preserve"> Problemi di truffa online            </t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>problemi_upgrade</t>
+          <t>problemi_sicurezza</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>0.7343999743461609</v>
+        <v>0.7210999727249146</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -618,20 +619,21 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>pagamenti_online pagamento_online confermare carta pausa pagamento attiva connessione riesce ogni</t>
+          <t xml:space="preserve"> Problemi di assistenza cliente
+             </t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>problemi_pagamenti_online</t>
+          <t>problemi_assistenza</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>0.7242000102996826</v>
+        <v>0.7026000022888184</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -641,20 +643,20 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>ultimo aggiornamento dopo apre chiude grazie riesco accedere appena problema</t>
+          <t xml:space="preserve"> Problemi di caricamenti.         </t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>problemi_upgrade</t>
+          <t>problemi_gestione_carta</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>0.6868000030517578</v>
+        <v>0.6861000061035156</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -664,20 +666,20 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>euro 25 50 10 bonus mese 250 pago 100 commissioni</t>
+          <t xml:space="preserve"> Problemi di accesso all'applic         </t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>problemi_concorsi_bonus</t>
+          <t>problemi_accesso</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>0.6223000288009644</v>
+        <v>0.6762999892234802</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -687,24 +689,212 @@
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>assistenza email mail carta chat dopo via problema giorni servizio</t>
+          <t xml:space="preserve"> Problemi di accesso all'applic         </t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
+          <t>problemi_accesso</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>0.6762999892234802</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Strong</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>11</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Problemi di costo elevato    
+         </t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>problemi_costi</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>0.6442000269889832</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Strong</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>6</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Problemi di registrazione online
+          Proble         </t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>problemi_registrazione</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>0.6399999856948853</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Strong</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>3</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Problemi di sicurezza
+                </t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>problemi_sicurezza</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>0.6133000254631042</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Strong</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>5</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Problemi di notifiche pubblicit         </t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
           <t>problemi_comunicazione</t>
         </is>
       </c>
-      <c r="D12" t="n">
-        <v>0.6201000213623047</v>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>Strong</t>
+      <c r="D16" t="n">
+        <v>0.603600025177002</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Strong</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>0</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Problemi di accesso
+        Return         </t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>problemi_accesso</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>0.5874000191688538</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Strong</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>12</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Problemi_di_pagamenti_e_assist         </t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>problemi_ricarica_telefonica</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>0.5529000163078308</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Strong</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>17</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Problemi di connessione internet.         </t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>problemi_ricarica_telefonica</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>0.5374000072479248</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Weak/New</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>8</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Problemi di velocità.         </t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>problemi_chiusura_conto</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>0.4133000075817108</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Weak/New</t>
         </is>
       </c>
     </row>

</xml_diff>